<commit_message>
change battle coefficients with card elements
</commit_message>
<xml_diff>
--- a/Assets/TypeChart.xlsx
+++ b/Assets/TypeChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CardGame\PokemonCardGame\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACFCCCED-1162-46E1-813A-F4CF45CF9C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E632C4-665E-41DE-8843-B393F69F7D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -669,7 +669,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="5">
         <v>1</v>
@@ -728,7 +728,7 @@
         <v>2</v>
       </c>
       <c r="M6" s="5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
@@ -757,7 +757,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5">
         <v>1</v>
@@ -789,7 +789,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G8" s="3">
         <v>0.5</v>
@@ -827,7 +827,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F9" s="6">
         <v>2</v>
@@ -985,7 +985,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="5">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D13" s="5">
         <v>1</v>

</xml_diff>

<commit_message>
add large set of intermediate changes
change project settings, UXML and USS files, change classes of mechanics, add new files and assets
</commit_message>
<xml_diff>
--- a/Assets/TypeChart.xlsx
+++ b/Assets/TypeChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CardGame\PokemonCardGame\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E632C4-665E-41DE-8843-B393F69F7D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC1A71E-7092-49D5-830F-05DF15A4FB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="14">
   <si>
     <t>Attacking \ Defending</t>
   </si>
@@ -39,9 +39,6 @@
     <t>Water</t>
   </si>
   <si>
-    <t>electric</t>
-  </si>
-  <si>
     <t>Bug</t>
   </si>
   <si>
@@ -64,6 +61,12 @@
   </si>
   <si>
     <t>Fairy</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Electric</t>
   </si>
 </sst>
 </file>
@@ -116,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -139,11 +142,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,6 +190,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -470,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -485,7 +529,7 @@
     <col min="13" max="13" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,34 +543,37 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -566,8 +613,11 @@
       <c r="M2" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N2" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -607,8 +657,11 @@
       <c r="M3" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N3" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -648,10 +701,13 @@
       <c r="M4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N4" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3">
         <v>0.5</v>
@@ -689,51 +745,57 @@
       <c r="M5" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N5" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K6" s="5">
+        <v>1</v>
+      </c>
+      <c r="L6" s="6">
+        <v>2</v>
+      </c>
+      <c r="M6" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="N6" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" s="6">
-        <v>2</v>
-      </c>
-      <c r="C6" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="D6" s="5">
-        <v>1</v>
-      </c>
-      <c r="E6" s="5">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5">
-        <v>1</v>
-      </c>
-      <c r="G6" s="5">
-        <v>1</v>
-      </c>
-      <c r="H6" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I6" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="K6" s="5">
-        <v>1</v>
-      </c>
-      <c r="L6" s="6">
-        <v>2</v>
-      </c>
-      <c r="M6" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>0.5</v>
@@ -771,255 +833,344 @@
       <c r="M7" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="N7" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6">
+        <v>2</v>
+      </c>
+      <c r="C8" s="5">
+        <v>1</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I8" s="5">
+        <v>1</v>
+      </c>
+      <c r="J8" s="5">
+        <v>1</v>
+      </c>
+      <c r="K8" s="5">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5">
+        <v>1</v>
+      </c>
+      <c r="M8" s="4">
+        <v>2</v>
+      </c>
+      <c r="N8" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6">
-        <v>2</v>
-      </c>
-      <c r="C8" s="5">
-        <v>1</v>
-      </c>
-      <c r="D8" s="5">
-        <v>1</v>
-      </c>
-      <c r="E8" s="5">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="H8" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I8" s="5">
-        <v>1</v>
-      </c>
-      <c r="J8" s="5">
-        <v>1</v>
-      </c>
-      <c r="K8" s="5">
-        <v>1</v>
-      </c>
-      <c r="L8" s="5">
-        <v>1</v>
-      </c>
-      <c r="M8" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="6">
+        <v>2</v>
+      </c>
+      <c r="C9" s="5">
+        <v>1</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="6">
+        <v>2</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
+      <c r="J9" s="6">
+        <v>2</v>
+      </c>
+      <c r="K9" s="5">
+        <v>1</v>
+      </c>
+      <c r="L9" s="5">
+        <v>1</v>
+      </c>
+      <c r="M9" s="5">
+        <v>1</v>
+      </c>
+      <c r="N9" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="6">
-        <v>2</v>
-      </c>
-      <c r="C9" s="5">
-        <v>1</v>
-      </c>
-      <c r="D9" s="5">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="F9" s="6">
-        <v>2</v>
-      </c>
-      <c r="G9" s="5">
-        <v>1</v>
-      </c>
-      <c r="H9" s="5">
-        <v>1</v>
-      </c>
-      <c r="I9" s="5">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6">
-        <v>2</v>
-      </c>
-      <c r="K9" s="5">
-        <v>1</v>
-      </c>
-      <c r="L9" s="5">
-        <v>1</v>
-      </c>
-      <c r="M9" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="5">
+        <v>1</v>
+      </c>
+      <c r="C10" s="5">
+        <v>1</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="J10" s="5">
+        <v>1</v>
+      </c>
+      <c r="K10" s="6">
+        <v>2</v>
+      </c>
+      <c r="L10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="N10" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5">
-        <v>1</v>
-      </c>
-      <c r="C10" s="5">
-        <v>1</v>
-      </c>
-      <c r="D10" s="5">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="G10" s="5">
-        <v>1</v>
-      </c>
-      <c r="H10" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I10" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="J10" s="5">
-        <v>1</v>
-      </c>
-      <c r="K10" s="6">
-        <v>2</v>
-      </c>
-      <c r="L10" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="M10" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5">
+        <v>1</v>
+      </c>
+      <c r="G11" s="5">
+        <v>1</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1</v>
+      </c>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+      <c r="J11" s="5">
+        <v>1</v>
+      </c>
+      <c r="K11" s="5">
+        <v>1</v>
+      </c>
+      <c r="L11" s="5">
+        <v>1</v>
+      </c>
+      <c r="M11" s="5">
+        <v>1</v>
+      </c>
+      <c r="N11" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="5">
-        <v>1</v>
-      </c>
-      <c r="C11" s="5">
-        <v>1</v>
-      </c>
-      <c r="D11" s="5">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5">
-        <v>1</v>
-      </c>
-      <c r="F11" s="5">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5">
-        <v>1</v>
-      </c>
-      <c r="H11" s="5">
-        <v>1</v>
-      </c>
-      <c r="I11" s="5">
-        <v>1</v>
-      </c>
-      <c r="J11" s="5">
-        <v>1</v>
-      </c>
-      <c r="K11" s="5">
-        <v>1</v>
-      </c>
-      <c r="L11" s="5">
-        <v>1</v>
-      </c>
-      <c r="M11" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="5">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1</v>
+      </c>
+      <c r="F12" s="5">
+        <v>1</v>
+      </c>
+      <c r="G12" s="5">
+        <v>1</v>
+      </c>
+      <c r="H12" s="6">
+        <v>2</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
+      <c r="J12" s="6">
+        <v>2</v>
+      </c>
+      <c r="K12" s="5">
+        <v>1</v>
+      </c>
+      <c r="L12" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M12" s="5">
+        <v>1</v>
+      </c>
+      <c r="N12" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="5">
-        <v>1</v>
-      </c>
-      <c r="C12" s="5">
-        <v>1</v>
-      </c>
-      <c r="D12" s="5">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5">
-        <v>1</v>
-      </c>
-      <c r="F12" s="5">
-        <v>1</v>
-      </c>
-      <c r="G12" s="5">
-        <v>1</v>
-      </c>
-      <c r="H12" s="6">
-        <v>2</v>
-      </c>
-      <c r="I12" s="5">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6">
-        <v>2</v>
-      </c>
-      <c r="K12" s="5">
-        <v>1</v>
-      </c>
-      <c r="L12" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="M12" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="8">
+        <v>1</v>
+      </c>
+      <c r="C13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="8">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8">
+        <v>1</v>
+      </c>
+      <c r="F13" s="8">
+        <v>1</v>
+      </c>
+      <c r="G13" s="8">
+        <v>1</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="8">
+        <v>1</v>
+      </c>
+      <c r="J13" s="10">
+        <v>2</v>
+      </c>
+      <c r="K13" s="8">
+        <v>1</v>
+      </c>
+      <c r="L13" s="8">
+        <v>1</v>
+      </c>
+      <c r="M13" s="8">
+        <v>1</v>
+      </c>
+      <c r="N13" s="11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5">
-        <v>1</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="5">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5">
-        <v>1</v>
-      </c>
-      <c r="F13" s="5">
-        <v>1</v>
-      </c>
-      <c r="G13" s="5">
-        <v>1</v>
-      </c>
-      <c r="H13" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I13" s="5">
-        <v>1</v>
-      </c>
-      <c r="J13" s="6">
-        <v>2</v>
-      </c>
-      <c r="K13" s="5">
-        <v>1</v>
-      </c>
-      <c r="L13" s="5">
-        <v>1</v>
-      </c>
-      <c r="M13" s="5">
-        <v>1</v>
+      <c r="B14" s="11">
+        <v>1</v>
+      </c>
+      <c r="C14" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="11">
+        <v>1</v>
+      </c>
+      <c r="G14" s="11">
+        <v>1</v>
+      </c>
+      <c r="H14" s="11">
+        <v>1</v>
+      </c>
+      <c r="I14" s="11">
+        <v>1</v>
+      </c>
+      <c r="J14" s="11">
+        <v>1</v>
+      </c>
+      <c r="K14" s="11">
+        <v>1</v>
+      </c>
+      <c r="L14" s="11">
+        <v>1</v>
+      </c>
+      <c r="M14" s="11">
+        <v>2</v>
+      </c>
+      <c r="N14" s="11">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:M13">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N14">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:N14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>